<commit_message>
feat: OOC template fix, pushed-tab for supervisor, duplicate-push guard, file split
- Replace leave-ooc.xlsx with user-provided template and update cell positions
  (D5=date, D9=days, H10=purpose, D16=name, D17=jobNum, D18=title, D19=date)
- Add canSeePushed = isAttendanceAdmin || isSupervisor so supervisor also sees
  the forwarded-leaves tab (fixes اختبار١ and gives supervisor visibility)
- Prevent duplicate pushToAdmin: guard returns early if req.pushedToAdmin is set
- Extract ApprovalsPage + InlineSigPad into ApprovalsPage.js (319 lines)
- UserPages.js reduced to 220 lines; Dashboard imports from new file
</commit_message>
<xml_diff>
--- a/public/templates/leave-ooc.xlsx
+++ b/public/templates/leave-ooc.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10625"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ihab1980\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{559119B2-598A-4035-A35E-7B1DFDA27AC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{22525E11-BA8F-7442-B9C0-5D26F1A1508B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1545" windowWidth="29040" windowHeight="15840" xr2:uid="{E7F8CA3B-B5D4-420F-B700-7FC7FF3FBA0B}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A$1:$I$43</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,9 +34,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -170,7 +167,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -467,7 +464,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1" readingOrder="2"/>
@@ -599,6 +596,12 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1004,20 +1007,20 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I44"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.28515625" customWidth="1"/>
-    <col min="2" max="2" width="14.42578125" customWidth="1"/>
-    <col min="3" max="3" width="16.5703125" customWidth="1"/>
-    <col min="4" max="4" width="16.28515625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="22.85546875" customWidth="1"/>
-    <col min="7" max="7" width="13.5703125" customWidth="1"/>
-    <col min="8" max="8" width="27.28515625" customWidth="1"/>
-    <col min="9" max="9" width="5.85546875" customWidth="1"/>
+    <col min="1" max="1" width="10.22265625" customWidth="1"/>
+    <col min="2" max="2" width="14.390625" customWidth="1"/>
+    <col min="3" max="3" width="16.54296875" customWidth="1"/>
+    <col min="4" max="4" width="16.27734375" customWidth="1"/>
+    <col min="5" max="5" width="11.97265625" customWidth="1"/>
+    <col min="6" max="6" width="22.8671875" customWidth="1"/>
+    <col min="7" max="7" width="13.5859375" customWidth="1"/>
+    <col min="8" max="8" width="27.3046875" customWidth="1"/>
+    <col min="9" max="9" width="5.91796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="32.25" customHeight="1" thickBot="1">
+    <row r="1" spans="1:9" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="38" t="s">
         <v>0</v>
       </c>
@@ -1036,7 +1039,7 @@
       </c>
       <c r="I1" s="41"/>
     </row>
-    <row r="2" spans="1:9" ht="36" customHeight="1" thickBot="1">
+    <row r="2" spans="1:9" ht="36" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="39"/>
       <c r="B2" s="44" t="s">
         <v>4</v>
@@ -1055,7 +1058,7 @@
       <c r="H2" s="42"/>
       <c r="I2" s="43"/>
     </row>
-    <row r="3" spans="1:9" ht="10.5" customHeight="1">
+    <row r="3" spans="1:9" ht="10.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
@@ -1065,7 +1068,7 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
     </row>
-    <row r="4" spans="1:9" ht="24.95" customHeight="1">
+    <row r="4" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4"/>
       <c r="B4" s="4"/>
       <c r="C4" s="20" t="s">
@@ -1082,7 +1085,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="24.95" customHeight="1">
+    <row r="5" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23"/>
       <c r="B5" s="23"/>
       <c r="C5" s="20" t="s">
@@ -1099,86 +1102,86 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="24.95" customHeight="1">
+    <row r="6" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B6" s="5"/>
     </row>
-    <row r="7" spans="1:9" ht="33" customHeight="1">
+    <row r="7" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
       <c r="F7" s="19" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="33" customHeight="1">
+    <row r="8" spans="1:9" ht="33" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
       <c r="F8" s="19"/>
     </row>
-    <row r="9" spans="1:9" ht="24.95" customHeight="1">
+    <row r="9" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="20"/>
       <c r="B9" s="22"/>
       <c r="C9" s="21" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="25" t="s">
+      <c r="F9" s="48" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:9" ht="24.95" customHeight="1">
+      <c r="G9" s="48"/>
+      <c r="H9" s="48"/>
+      <c r="I9" s="48"/>
+    </row>
+    <row r="10" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="22"/>
       <c r="B10" s="22"/>
       <c r="C10" s="20"/>
       <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20" t="s">
+      <c r="E10" s="49" t="s">
         <v>25</v>
       </c>
+      <c r="F10" s="49"/>
+      <c r="G10" s="49"/>
       <c r="H10" s="20"/>
       <c r="I10" s="22" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="24.95" customHeight="1">
+    <row r="11" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="7"/>
       <c r="B11" s="7"/>
     </row>
-    <row r="12" spans="1:9" ht="24.95" customHeight="1">
+    <row r="12" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
     </row>
-    <row r="13" spans="1:9" ht="24.95" customHeight="1">
+    <row r="13" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="7"/>
       <c r="B13" s="7"/>
       <c r="E13" s="10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="24.95" customHeight="1">
+    <row r="14" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
       <c r="B14" s="9"/>
     </row>
-    <row r="15" spans="1:9" ht="24.95" customHeight="1">
+    <row r="15" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="10"/>
       <c r="C15" s="25" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:9" ht="24.95" customHeight="1">
+    <row r="16" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="11"/>
       <c r="B16" s="11"/>
       <c r="C16" s="25" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="17" spans="1:9" ht="24.95" customHeight="1">
+    <row r="17" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="12" t="s">
         <v>10</v>
       </c>
@@ -1187,51 +1190,51 @@
         <v>29</v>
       </c>
     </row>
-    <row r="18" spans="1:9" ht="24.95" customHeight="1">
+    <row r="18" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="25" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="19" spans="1:9" ht="24.95" customHeight="1">
+    <row r="19" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="14"/>
       <c r="B19" s="14"/>
       <c r="C19" s="25" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="20" spans="1:9" ht="24.95" customHeight="1">
+    <row r="20" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14"/>
       <c r="B20" s="14"/>
     </row>
-    <row r="21" spans="1:9" ht="24.95" customHeight="1">
+    <row r="21" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="15" t="s">
         <v>0</v>
       </c>
       <c r="B21" s="15"/>
     </row>
-    <row r="22" spans="1:9" ht="24.95" customHeight="1">
+    <row r="22" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="16"/>
       <c r="B22" s="16"/>
     </row>
-    <row r="23" spans="1:9" ht="24.95" customHeight="1">
+    <row r="23" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="16"/>
       <c r="B23" s="16"/>
     </row>
-    <row r="24" spans="1:9" ht="24.95" customHeight="1">
+    <row r="24" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
     </row>
-    <row r="25" spans="1:9" ht="24.95" customHeight="1">
+    <row r="25" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="16"/>
       <c r="B25" s="16"/>
     </row>
-    <row r="26" spans="1:9" ht="24.95" customHeight="1">
+    <row r="26" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="16"/>
       <c r="B26" s="16"/>
     </row>
-    <row r="27" spans="1:9" ht="24.95" customHeight="1">
+    <row r="27" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="24"/>
       <c r="B27" s="25"/>
       <c r="C27" s="26" t="s">
@@ -1248,7 +1251,7 @@
       </c>
       <c r="I27" s="25"/>
     </row>
-    <row r="28" spans="1:9" ht="24.95" customHeight="1">
+    <row r="28" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="25"/>
       <c r="B28" s="28"/>
       <c r="C28" s="25"/>
@@ -1259,7 +1262,7 @@
       <c r="H28" s="25"/>
       <c r="I28" s="25"/>
     </row>
-    <row r="29" spans="1:9" ht="24.95" customHeight="1">
+    <row r="29" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="28"/>
       <c r="B29" s="28"/>
       <c r="C29" s="25"/>
@@ -1270,7 +1273,7 @@
       <c r="H29" s="25"/>
       <c r="I29" s="25"/>
     </row>
-    <row r="30" spans="1:9" ht="24.95" customHeight="1">
+    <row r="30" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="28"/>
       <c r="B30" s="28"/>
       <c r="C30" s="29" t="s">
@@ -1283,7 +1286,7 @@
       <c r="H30" s="25"/>
       <c r="I30" s="25"/>
     </row>
-    <row r="31" spans="1:9" ht="24.95" customHeight="1">
+    <row r="31" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="30" t="s">
         <v>11</v>
       </c>
@@ -1296,7 +1299,7 @@
       <c r="H31" s="25"/>
       <c r="I31" s="25"/>
     </row>
-    <row r="32" spans="1:9" ht="24.95" customHeight="1">
+    <row r="32" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="31"/>
       <c r="B32" s="31"/>
       <c r="C32" s="25"/>
@@ -1307,7 +1310,7 @@
       <c r="H32" s="25"/>
       <c r="I32" s="25"/>
     </row>
-    <row r="33" spans="1:9" ht="24.95" customHeight="1">
+    <row r="33" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="35" t="s">
         <v>36</v>
       </c>
@@ -1320,7 +1323,7 @@
       <c r="H33" s="36"/>
       <c r="I33" s="37"/>
     </row>
-    <row r="34" spans="1:9" ht="24.95" customHeight="1">
+    <row r="34" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="32"/>
       <c r="B34" s="32"/>
       <c r="C34" s="32"/>
@@ -1331,7 +1334,7 @@
       <c r="H34" s="32"/>
       <c r="I34" s="32"/>
     </row>
-    <row r="35" spans="1:9" ht="24.95" customHeight="1">
+    <row r="35" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="25"/>
       <c r="B35" s="17"/>
       <c r="C35" s="25"/>
@@ -1344,7 +1347,7 @@
       <c r="H35" s="25"/>
       <c r="I35" s="25"/>
     </row>
-    <row r="36" spans="1:9" ht="24.95" customHeight="1">
+    <row r="36" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="33"/>
       <c r="B36" s="33"/>
       <c r="C36" s="25"/>
@@ -1355,7 +1358,7 @@
       <c r="H36" s="25"/>
       <c r="I36" s="25"/>
     </row>
-    <row r="37" spans="1:9" ht="24.95" customHeight="1">
+    <row r="37" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="25"/>
       <c r="B37" s="28"/>
       <c r="C37" s="25"/>
@@ -1368,7 +1371,7 @@
       </c>
       <c r="I37" s="25"/>
     </row>
-    <row r="38" spans="1:9" ht="24.95" customHeight="1">
+    <row r="38" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="25"/>
       <c r="B38" s="33"/>
       <c r="C38" s="25"/>
@@ -1379,7 +1382,7 @@
       <c r="H38" s="25"/>
       <c r="I38" s="25"/>
     </row>
-    <row r="39" spans="1:9" ht="24.95" customHeight="1">
+    <row r="39" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="33"/>
       <c r="B39" s="33"/>
       <c r="C39" s="25"/>
@@ -1392,7 +1395,7 @@
       <c r="H39" s="25"/>
       <c r="I39" s="25"/>
     </row>
-    <row r="40" spans="1:9" ht="24.95" customHeight="1">
+    <row r="40" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="33"/>
       <c r="B40" s="33"/>
       <c r="C40" s="25"/>
@@ -1403,7 +1406,7 @@
       <c r="H40" s="25"/>
       <c r="I40" s="25"/>
     </row>
-    <row r="41" spans="1:9" ht="24.95" customHeight="1">
+    <row r="41" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="33"/>
       <c r="B41" s="33"/>
       <c r="C41" s="25"/>
@@ -1414,7 +1417,7 @@
       <c r="H41" s="25"/>
       <c r="I41" s="25"/>
     </row>
-    <row r="42" spans="1:9" ht="24.95" customHeight="1">
+    <row r="42" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="33"/>
       <c r="B42" s="34" t="s">
         <v>15</v>
@@ -1427,7 +1430,7 @@
       <c r="H42" s="25"/>
       <c r="I42" s="25"/>
     </row>
-    <row r="43" spans="1:9" ht="24.95" customHeight="1">
+    <row r="43" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="33"/>
       <c r="B43" s="33"/>
       <c r="C43" s="25"/>
@@ -1438,7 +1441,7 @@
       <c r="H43" s="25"/>
       <c r="I43" s="25"/>
     </row>
-    <row r="44" spans="1:9" ht="24.95" customHeight="1">
+    <row r="44" spans="1:9" ht="24.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="25"/>
       <c r="B44" s="34"/>
       <c r="C44" s="25"/>
@@ -1450,13 +1453,15 @@
       <c r="I44" s="25"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A33:I33"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="H1:I2"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="E10:G10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="62" orientation="portrait" r:id="rId1"/>

</xml_diff>